<commit_message>
Working on dataset loaders
- Loading in survey data
- Generating labels based on HRV times
</commit_message>
<xml_diff>
--- a/software/python_processing/dataset_stats/cLASIr Dataset Binary Stats.xlsx
+++ b/software/python_processing/dataset_stats/cLASIr Dataset Binary Stats.xlsx
@@ -452,7 +452,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>214</v>
+        <v>754</v>
       </c>
       <c r="C2" t="n">
         <v>972</v>
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>322</v>
+        <v>1036</v>
       </c>
       <c r="C3" t="n">
         <v>1138</v>
@@ -478,7 +478,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>236</v>
+        <v>736</v>
       </c>
       <c r="C4" t="n">
         <v>904</v>
@@ -491,7 +491,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>228</v>
+        <v>740</v>
       </c>
       <c r="C5" t="n">
         <v>890</v>
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>200</v>
+        <v>772</v>
       </c>
       <c r="C6" t="n">
         <v>998</v>
@@ -517,7 +517,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>180</v>
+        <v>547</v>
       </c>
       <c r="C7" t="n">
         <v>904</v>
@@ -530,7 +530,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>234</v>
+        <v>818</v>
       </c>
       <c r="C8" t="n">
         <v>1298</v>
@@ -543,7 +543,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>294</v>
+        <v>744</v>
       </c>
       <c r="C9" t="n">
         <v>960</v>
@@ -556,7 +556,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>264</v>
+        <v>734</v>
       </c>
       <c r="C10" t="n">
         <v>972</v>
@@ -569,7 +569,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>384</v>
+        <v>882</v>
       </c>
       <c r="C11" t="n">
         <v>954</v>
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>262</v>
+        <v>786</v>
       </c>
       <c r="C12" t="n">
         <v>1008</v>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>230</v>
+        <v>712</v>
       </c>
       <c r="C13" t="n">
         <v>886</v>
@@ -608,7 +608,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>222</v>
+        <v>934</v>
       </c>
       <c r="C14" t="n">
         <v>950</v>
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>242</v>
+        <v>894</v>
       </c>
       <c r="C15" t="n">
         <v>976</v>
@@ -634,7 +634,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>290</v>
+        <v>739</v>
       </c>
       <c r="C16" t="n">
         <v>859</v>
@@ -647,7 +647,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>226</v>
+        <v>730</v>
       </c>
       <c r="C17" t="n">
         <v>920</v>
@@ -660,7 +660,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>232</v>
+        <v>766</v>
       </c>
       <c r="C18" t="n">
         <v>926</v>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>214</v>
+        <v>812</v>
       </c>
       <c r="C19" t="n">
         <v>1026</v>
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>246</v>
+        <v>738</v>
       </c>
       <c r="C20" t="n">
         <v>938</v>
@@ -699,7 +699,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>224</v>
+        <v>660</v>
       </c>
       <c r="C21" t="n">
         <v>886</v>
@@ -712,7 +712,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>254</v>
+        <v>726</v>
       </c>
       <c r="C22" t="n">
         <v>856</v>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>212</v>
+        <v>818</v>
       </c>
       <c r="C23" t="n">
         <v>952</v>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>208</v>
+        <v>744</v>
       </c>
       <c r="C24" t="n">
         <v>950</v>
@@ -751,7 +751,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>232</v>
+        <v>794</v>
       </c>
       <c r="C25" t="n">
         <v>902</v>
@@ -764,7 +764,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>232</v>
+        <v>804</v>
       </c>
       <c r="C26" t="n">
         <v>916</v>
@@ -777,7 +777,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>246</v>
+        <v>702</v>
       </c>
       <c r="C27" t="n">
         <v>956</v>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>216</v>
+        <v>730</v>
       </c>
       <c r="C28" t="n">
         <v>914</v>
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>266</v>
+        <v>656</v>
       </c>
       <c r="C29" t="n">
         <v>876</v>
@@ -816,7 +816,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>228</v>
+        <v>852</v>
       </c>
       <c r="C30" t="n">
         <v>1088</v>
@@ -829,7 +829,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>246</v>
+        <v>782</v>
       </c>
       <c r="C31" t="n">
         <v>916</v>
@@ -842,7 +842,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>242</v>
+        <v>794</v>
       </c>
       <c r="C32" t="n">
         <v>962</v>
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>230</v>
+        <v>866</v>
       </c>
       <c r="C33" t="n">
         <v>1094</v>
@@ -868,7 +868,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>254</v>
+        <v>746</v>
       </c>
       <c r="C34" t="n">
         <v>936</v>
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>246</v>
+        <v>666</v>
       </c>
       <c r="C35" t="n">
         <v>868</v>
@@ -894,7 +894,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>230</v>
+        <v>806</v>
       </c>
       <c r="C36" t="n">
         <v>1016</v>
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>254</v>
+        <v>760</v>
       </c>
       <c r="C37" t="n">
         <v>1144</v>
@@ -920,7 +920,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>242</v>
+        <v>704</v>
       </c>
       <c r="C38" t="n">
         <v>862</v>
@@ -933,7 +933,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>260</v>
+        <v>746</v>
       </c>
       <c r="C39" t="n">
         <v>950</v>
@@ -946,7 +946,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>234</v>
+        <v>718</v>
       </c>
       <c r="C40" t="n">
         <v>928</v>
@@ -959,7 +959,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>230</v>
+        <v>748</v>
       </c>
       <c r="C41" t="n">
         <v>1016</v>
@@ -972,7 +972,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>210</v>
+        <v>792</v>
       </c>
       <c r="C42" t="n">
         <v>1090</v>
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>234</v>
+        <v>800</v>
       </c>
       <c r="C43" t="n">
         <v>1044</v>
@@ -998,7 +998,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>220</v>
+        <v>796</v>
       </c>
       <c r="C44" t="n">
         <v>1004</v>
@@ -1011,7 +1011,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>224</v>
+        <v>754</v>
       </c>
       <c r="C45" t="n">
         <v>910</v>
@@ -1024,7 +1024,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>232</v>
+        <v>786</v>
       </c>
       <c r="C46" t="n">
         <v>1034</v>
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>239</v>
+        <v>765</v>
       </c>
       <c r="C47" t="n">
         <v>950</v>
@@ -1050,7 +1050,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>226</v>
+        <v>692</v>
       </c>
       <c r="C48" t="n">
         <v>952</v>
@@ -1063,7 +1063,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>224</v>
+        <v>858</v>
       </c>
       <c r="C49" t="n">
         <v>1078</v>
@@ -1076,7 +1076,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>248</v>
+        <v>708</v>
       </c>
       <c r="C50" t="n">
         <v>994</v>
@@ -1089,7 +1089,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>248</v>
+        <v>806</v>
       </c>
       <c r="C51" t="n">
         <v>676</v>
@@ -1102,7 +1102,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>232</v>
+        <v>828</v>
       </c>
       <c r="C52" t="n">
         <v>1182</v>
@@ -1115,7 +1115,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>222</v>
+        <v>812</v>
       </c>
       <c r="C53" t="n">
         <v>1030</v>
@@ -1128,7 +1128,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>232</v>
+        <v>862</v>
       </c>
       <c r="C54" t="n">
         <v>1031</v>
@@ -1141,7 +1141,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>242</v>
+        <v>840</v>
       </c>
       <c r="C55" t="n">
         <v>1088</v>
@@ -1154,7 +1154,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>288</v>
+        <v>744</v>
       </c>
       <c r="C56" t="n">
         <v>884</v>
@@ -1167,7 +1167,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>212</v>
+        <v>788</v>
       </c>
       <c r="C57" t="n">
         <v>990</v>
@@ -1180,7 +1180,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>257</v>
+        <v>689</v>
       </c>
       <c r="C58" t="n">
         <v>914</v>
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>276</v>
+        <v>702</v>
       </c>
       <c r="C59" t="n">
         <v>822</v>
@@ -1206,7 +1206,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>160</v>
+        <v>754</v>
       </c>
       <c r="C60" t="n">
         <v>970</v>
@@ -1219,7 +1219,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>242</v>
+        <v>672</v>
       </c>
       <c r="C61" t="n">
         <v>850</v>
@@ -1232,7 +1232,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>210</v>
+        <v>952</v>
       </c>
       <c r="C62" t="n">
         <v>972</v>
@@ -1245,7 +1245,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>216</v>
+        <v>830</v>
       </c>
       <c r="C63" t="n">
         <v>982</v>
@@ -1258,7 +1258,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>208</v>
+        <v>758</v>
       </c>
       <c r="C64" t="n">
         <v>1048</v>
@@ -1271,7 +1271,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>292</v>
+        <v>830</v>
       </c>
       <c r="C65" t="n">
         <v>982</v>
@@ -1284,7 +1284,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>214</v>
+        <v>740</v>
       </c>
       <c r="C66" t="n">
         <v>938</v>
@@ -1297,7 +1297,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>230</v>
+        <v>814</v>
       </c>
       <c r="C67" t="n">
         <v>1100</v>
@@ -1310,7 +1310,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>206</v>
+        <v>708</v>
       </c>
       <c r="C68" t="n">
         <v>928</v>
@@ -1323,7 +1323,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>224</v>
+        <v>508</v>
       </c>
       <c r="C69" t="n">
         <v>1080</v>
@@ -1336,7 +1336,7 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>312</v>
+        <v>734</v>
       </c>
       <c r="C70" t="n">
         <v>1046</v>
@@ -1349,7 +1349,7 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>214</v>
+        <v>882</v>
       </c>
       <c r="C71" t="n">
         <v>1024</v>
@@ -1362,7 +1362,7 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>230</v>
+        <v>740</v>
       </c>
       <c r="C72" t="n">
         <v>1170</v>
@@ -1375,7 +1375,7 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>212</v>
+        <v>750</v>
       </c>
       <c r="C73" t="n">
         <v>1138</v>
@@ -1388,7 +1388,7 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>230</v>
+        <v>826</v>
       </c>
       <c r="C74" t="n">
         <v>1278</v>
@@ -1401,7 +1401,7 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>232</v>
+        <v>806</v>
       </c>
       <c r="C75" t="n">
         <v>1104</v>
@@ -1414,7 +1414,7 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>236</v>
+        <v>774</v>
       </c>
       <c r="C76" t="n">
         <v>1090</v>
@@ -1427,7 +1427,7 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>212</v>
+        <v>800</v>
       </c>
       <c r="C77" t="n">
         <v>1186</v>
@@ -1440,7 +1440,7 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>254</v>
+        <v>814</v>
       </c>
       <c r="C78" t="n">
         <v>1176</v>
@@ -1453,7 +1453,7 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>214</v>
+        <v>802</v>
       </c>
       <c r="C79" t="n">
         <v>1022</v>
@@ -1466,7 +1466,7 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>244</v>
+        <v>732</v>
       </c>
       <c r="C80" t="n">
         <v>1144</v>
@@ -1479,7 +1479,7 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>276</v>
+        <v>727</v>
       </c>
       <c r="C81" t="n">
         <v>1136</v>
@@ -1492,7 +1492,7 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>228</v>
+        <v>762</v>
       </c>
       <c r="C82" t="n">
         <v>1110</v>
@@ -1505,7 +1505,7 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>214</v>
+        <v>902</v>
       </c>
       <c r="C83" t="n">
         <v>1370</v>
@@ -1518,7 +1518,7 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>270</v>
+        <v>768</v>
       </c>
       <c r="C84" t="n">
         <v>1050</v>
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>214</v>
+        <v>782</v>
       </c>
       <c r="C85" t="n">
         <v>1100</v>
@@ -1544,7 +1544,7 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>234</v>
+        <v>696</v>
       </c>
       <c r="C86" t="n">
         <v>1000</v>
@@ -1557,7 +1557,7 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>212</v>
+        <v>854</v>
       </c>
       <c r="C87" t="n">
         <v>1078</v>
@@ -1570,7 +1570,7 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>264</v>
+        <v>816</v>
       </c>
       <c r="C88" t="n">
         <v>1392</v>
@@ -1583,7 +1583,7 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>214</v>
+        <v>798</v>
       </c>
       <c r="C89" t="n">
         <v>1266</v>
@@ -1596,7 +1596,7 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>288</v>
+        <v>715</v>
       </c>
       <c r="C90" t="n">
         <v>1004</v>
@@ -1609,7 +1609,7 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>220</v>
+        <v>758</v>
       </c>
       <c r="C91" t="n">
         <v>1156</v>
@@ -1622,7 +1622,7 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>216</v>
+        <v>794</v>
       </c>
       <c r="C92" t="n">
         <v>1280</v>
@@ -1635,7 +1635,7 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>234</v>
+        <v>848</v>
       </c>
       <c r="C93" t="n">
         <v>1212</v>
@@ -1648,7 +1648,7 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>220</v>
+        <v>744</v>
       </c>
       <c r="C94" t="n">
         <v>1319</v>
@@ -1661,7 +1661,7 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>229</v>
+        <v>804</v>
       </c>
       <c r="C95" t="n">
         <v>1057</v>
@@ -1674,7 +1674,7 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>216</v>
+        <v>796</v>
       </c>
       <c r="C96" t="n">
         <v>1280</v>
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>234</v>
+        <v>763</v>
       </c>
       <c r="C97" t="n">
         <v>1145</v>
@@ -1700,7 +1700,7 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>250</v>
+        <v>883</v>
       </c>
       <c r="C98" t="n">
         <v>1360</v>
@@ -1713,7 +1713,7 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>250</v>
+        <v>772</v>
       </c>
       <c r="C99" t="n">
         <v>1158</v>
@@ -1726,7 +1726,7 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>225</v>
+        <v>846</v>
       </c>
       <c r="C100" t="n">
         <v>1349</v>
@@ -1739,7 +1739,7 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>293</v>
+        <v>722</v>
       </c>
       <c r="C101" t="n">
         <v>1053</v>
@@ -1752,7 +1752,7 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>275</v>
+        <v>915</v>
       </c>
       <c r="C102" t="n">
         <v>1332</v>
@@ -1765,7 +1765,7 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>290</v>
+        <v>758</v>
       </c>
       <c r="C103" t="n">
         <v>1132</v>
@@ -1778,7 +1778,7 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>238</v>
+        <v>763</v>
       </c>
       <c r="C104" t="n">
         <v>1159</v>
@@ -1791,7 +1791,7 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>235</v>
+        <v>883</v>
       </c>
       <c r="C105" t="n">
         <v>1251</v>
@@ -1804,7 +1804,7 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>211</v>
+        <v>730</v>
       </c>
       <c r="C106" t="n">
         <v>1227</v>
@@ -1817,7 +1817,7 @@
         </is>
       </c>
       <c r="B107" t="n">
-        <v>215</v>
+        <v>834</v>
       </c>
       <c r="C107" t="n">
         <v>1239</v>
@@ -1830,7 +1830,7 @@
         </is>
       </c>
       <c r="B108" t="n">
-        <v>256</v>
+        <v>738</v>
       </c>
       <c r="C108" t="n">
         <v>960</v>
@@ -1843,7 +1843,7 @@
         </is>
       </c>
       <c r="B109" t="n">
-        <v>247</v>
+        <v>735</v>
       </c>
       <c r="C109" t="n">
         <v>1141</v>
@@ -1856,7 +1856,7 @@
         </is>
       </c>
       <c r="B110" t="n">
-        <v>224</v>
+        <v>777</v>
       </c>
       <c r="C110" t="n">
         <v>1173</v>
@@ -1869,7 +1869,7 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>209</v>
+        <v>774</v>
       </c>
       <c r="C111" t="n">
         <v>1162</v>
@@ -1882,7 +1882,7 @@
         </is>
       </c>
       <c r="B112" t="n">
-        <v>237</v>
+        <v>821</v>
       </c>
       <c r="C112" t="n">
         <v>1121</v>
@@ -1895,7 +1895,7 @@
         </is>
       </c>
       <c r="B113" t="n">
-        <v>207</v>
+        <v>755</v>
       </c>
       <c r="C113" t="n">
         <v>1128</v>
@@ -1908,7 +1908,7 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>236</v>
+        <v>1019</v>
       </c>
       <c r="C114" t="n">
         <v>1428</v>
@@ -1921,7 +1921,7 @@
         </is>
       </c>
       <c r="B115" t="n">
-        <v>205</v>
+        <v>809</v>
       </c>
       <c r="C115" t="n">
         <v>1231</v>
@@ -1934,7 +1934,7 @@
         </is>
       </c>
       <c r="B116" t="n">
-        <v>223</v>
+        <v>780</v>
       </c>
       <c r="C116" t="n">
         <v>1247</v>
@@ -1947,7 +1947,7 @@
         </is>
       </c>
       <c r="B117" t="n">
-        <v>215</v>
+        <v>1000</v>
       </c>
       <c r="C117" t="n">
         <v>1253</v>
@@ -1960,7 +1960,7 @@
         </is>
       </c>
       <c r="B118" t="n">
-        <v>339</v>
+        <v>703</v>
       </c>
       <c r="C118" t="n">
         <v>1006</v>
@@ -1973,7 +1973,7 @@
         </is>
       </c>
       <c r="B119" t="n">
-        <v>222</v>
+        <v>767</v>
       </c>
       <c r="C119" t="n">
         <v>1077</v>
@@ -1986,7 +1986,7 @@
         </is>
       </c>
       <c r="B120" t="n">
-        <v>233</v>
+        <v>806</v>
       </c>
       <c r="C120" t="n">
         <v>1221</v>
@@ -1999,7 +1999,7 @@
         </is>
       </c>
       <c r="B121" t="n">
-        <v>249</v>
+        <v>810</v>
       </c>
       <c r="C121" t="n">
         <v>1005</v>
@@ -2012,7 +2012,7 @@
         </is>
       </c>
       <c r="B122" t="n">
-        <v>303</v>
+        <v>735</v>
       </c>
       <c r="C122" t="n">
         <v>1084</v>
@@ -2025,7 +2025,7 @@
         </is>
       </c>
       <c r="B123" t="n">
-        <v>214</v>
+        <v>859</v>
       </c>
       <c r="C123" t="n">
         <v>1469</v>
@@ -2038,7 +2038,7 @@
         </is>
       </c>
       <c r="B124" t="n">
-        <v>367</v>
+        <v>743</v>
       </c>
       <c r="C124" t="n">
         <v>1067</v>
@@ -2051,7 +2051,7 @@
         </is>
       </c>
       <c r="B125" t="n">
-        <v>271</v>
+        <v>688</v>
       </c>
       <c r="C125" t="n">
         <v>1076</v>
@@ -2064,7 +2064,7 @@
         </is>
       </c>
       <c r="B126" t="n">
-        <v>275</v>
+        <v>880</v>
       </c>
       <c r="C126" t="n">
         <v>1124</v>
@@ -2077,7 +2077,7 @@
         </is>
       </c>
       <c r="B127" t="n">
-        <v>347</v>
+        <v>859</v>
       </c>
       <c r="C127" t="n">
         <v>1105</v>
@@ -2090,7 +2090,7 @@
         </is>
       </c>
       <c r="B128" t="n">
-        <v>334</v>
+        <v>685</v>
       </c>
       <c r="C128" t="n">
         <v>984</v>
@@ -2103,7 +2103,7 @@
         </is>
       </c>
       <c r="B129" t="n">
-        <v>331</v>
+        <v>765</v>
       </c>
       <c r="C129" t="n">
         <v>1168</v>
@@ -2116,7 +2116,7 @@
         </is>
       </c>
       <c r="B130" t="n">
-        <v>214</v>
+        <v>834</v>
       </c>
       <c r="C130" t="n">
         <v>1202</v>
@@ -2129,7 +2129,7 @@
         </is>
       </c>
       <c r="B131" t="n">
-        <v>298</v>
+        <v>749</v>
       </c>
       <c r="C131" t="n">
         <v>1011</v>
@@ -2142,7 +2142,7 @@
         </is>
       </c>
       <c r="B132" t="n">
-        <v>234</v>
+        <v>14</v>
       </c>
       <c r="C132" t="n">
         <v>1164</v>
@@ -2155,7 +2155,7 @@
         </is>
       </c>
       <c r="B133" t="n">
-        <v>145</v>
+        <v>819</v>
       </c>
       <c r="C133" t="n">
         <v>1207</v>
@@ -2168,7 +2168,7 @@
         </is>
       </c>
       <c r="B134" t="n">
-        <v>216</v>
+        <v>857</v>
       </c>
       <c r="C134" t="n">
         <v>1202</v>
@@ -2181,7 +2181,7 @@
         </is>
       </c>
       <c r="B135" t="n">
-        <v>328</v>
+        <v>689</v>
       </c>
       <c r="C135" t="n">
         <v>938</v>
@@ -2194,7 +2194,7 @@
         </is>
       </c>
       <c r="B136" t="n">
-        <v>142</v>
+        <v>856</v>
       </c>
       <c r="C136" t="n">
         <v>1013</v>
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="B137" t="n">
-        <v>301</v>
+        <v>964</v>
       </c>
       <c r="C137" t="n">
         <v>1347</v>
@@ -2220,7 +2220,7 @@
         </is>
       </c>
       <c r="B138" t="n">
-        <v>210</v>
+        <v>816</v>
       </c>
       <c r="C138" t="n">
         <v>1118</v>
@@ -2233,7 +2233,7 @@
         </is>
       </c>
       <c r="B139" t="n">
-        <v>454</v>
+        <v>849</v>
       </c>
       <c r="C139" t="n">
         <v>1244</v>
@@ -2246,7 +2246,7 @@
         </is>
       </c>
       <c r="B140" t="n">
-        <v>306</v>
+        <v>767</v>
       </c>
       <c r="C140" t="n">
         <v>1090</v>
@@ -2259,7 +2259,7 @@
         </is>
       </c>
       <c r="B141" t="n">
-        <v>207</v>
+        <v>718</v>
       </c>
       <c r="C141" t="n">
         <v>1007</v>

</xml_diff>